<commit_message>
[fix] Text Legacy를 TextMeshPro로 변경
Text Legacy를 TextMeshPro로 변경
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Entity.xlsx
+++ b/JsonConverter/ExcelFiles/Entity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\MinHyeong2DProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD49A0B-6ADD-488D-B8D2-9E49F7749E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86166028-B2C1-49D3-A752-71E894D51953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -218,27 +218,27 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>독침을 이용해 적의 방어력을 감소시키는 원시인\n지상과 공중 유닛을 공격할 수 있습니다.</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>창을 이용해 적을 찌르는 원시인\n날아다니는 유닛을 공격할 수 없습니다.</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>도끼를 이용해 적을 공격하는 원시인\n날아다니는 유닛을 공격할 수 없습니다.</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>돌을 던져 먼 거리에서 공격할 수 있는 원시인\n지상과 공중 유닛을 공격할 수 있습니다.</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>화살을 이용해 먼 거리를 강력하게 공격할 수 있는 원시인\n지상과 공중 유닛을 공격할 수 있습니다.</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>밧줄을 던져 적의 이동속도를 감소시키는 원시인\n지상과 공중 유닛을 공격할 수 있습니다.</t>
+    <t>창을 이용해 적을 찌르는 원시인&lt;br&gt;날아다니는 유닛을 공격할 수 없습니다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>도끼를 이용해 적을 공격하는 원시인&lt;br&gt;날아다니는 유닛을 공격할 수 없습니다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>돌을 던져 먼 거리에서 공격할 수 있는 원시인&lt;br&gt;지상과 공중 유닛을 공격할 수 있습니다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>화살을 이용해 먼 거리를 강력하게 공격할 수 있는 원시인&lt;br&gt;지상과 공중 유닛을 공격할 수 있습니다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>독침을 이용해 적의 방어력을 감소시키는 원시인&lt;br&gt;지상과 공중 유닛을 공격할 수 있습니다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>밧줄을 던져 적의 이동속도를 감소시키는 원시인&lt;br&gt;지상과 공중 유닛을 공격할 수 있습니다.</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -395,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -434,6 +434,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -738,8 +741,8 @@
       <c r="B4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>51</v>
+      <c r="C4" s="22" t="s">
+        <v>50</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>12</v>
@@ -766,7 +769,7 @@
         <v>24</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>12</v>
@@ -793,7 +796,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>12</v>
@@ -820,7 +823,7 @@
         <v>29</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>12</v>
@@ -847,7 +850,7 @@
         <v>30</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>12</v>

</xml_diff>